<commit_message>
new graphs and t-tests
</commit_message>
<xml_diff>
--- a/UTh and MeCa combined sediment pteropods.xlsx
+++ b/UTh and MeCa combined sediment pteropods.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/clairesheppard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/clairesheppard/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{519B34C5-708F-3B4E-A323-B3D2E8F72748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AF2BC50-DD0D-474B-B892-882C0C61EF50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8640" yWindow="2260" windowWidth="20080" windowHeight="15740" activeTab="2" xr2:uid="{F4C862C2-342B-0B41-8C63-E12B64784535}"/>
+    <workbookView xWindow="8640" yWindow="2260" windowWidth="20080" windowHeight="15740" xr2:uid="{F4C862C2-342B-0B41-8C63-E12B64784535}"/>
   </bookViews>
   <sheets>
     <sheet name="combined sedimentary pteropods" sheetId="1" r:id="rId1"/>
@@ -19,10 +19,10 @@
     <sheet name="unit conversion" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">('workup for cleaning types'!$X$12,'workup for cleaning types'!$X$14)</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">('workup for cleaning types'!$X$3,'workup for cleaning types'!$X$5)</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">('workup for cleaning types'!$X$7,'workup for cleaning types'!$X$8)</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">('workup for cleaning types'!$X$9,'workup for cleaning types'!$X$10,'workup for cleaning types'!$X$11)</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">('workup for cleaning types'!$Y$12,'workup for cleaning types'!$Y$14)</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">('workup for cleaning types'!$Y$3,'workup for cleaning types'!$Y$5)</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">('workup for cleaning types'!$Y$7,'workup for cleaning types'!$Y$8)</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">('workup for cleaning types'!$Y$9,'workup for cleaning types'!$Y$10,'workup for cleaning types'!$Y$11)</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="69">
   <si>
     <t>Sediment</t>
   </si>
@@ -271,6 +271,9 @@
   </si>
   <si>
     <t>sonic++red+ox</t>
+  </si>
+  <si>
+    <t>number</t>
   </si>
 </sst>
 </file>
@@ -546,7 +549,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>('combined sedimentary pteropods'!$X$3,'combined sedimentary pteropods'!$X$5,'combined sedimentary pteropods'!$X$7:$X$12,'combined sedimentary pteropods'!$X$14)</c:f>
+              <c:f>('combined sedimentary pteropods'!$Y$3,'combined sedimentary pteropods'!$Y$5,'combined sedimentary pteropods'!$Y$7:$Y$12,'combined sedimentary pteropods'!$Y$14)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -582,7 +585,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>('combined sedimentary pteropods'!$AB$3,'combined sedimentary pteropods'!$AB$5,'combined sedimentary pteropods'!$AB$7:$AB$12,'combined sedimentary pteropods'!$AB$14)</c:f>
+              <c:f>('combined sedimentary pteropods'!$AC$3,'combined sedimentary pteropods'!$AC$5,'combined sedimentary pteropods'!$AC$7:$AC$12,'combined sedimentary pteropods'!$AC$14)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -1046,7 +1049,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>('combined sedimentary pteropods'!$X$3,'combined sedimentary pteropods'!$X$5)</c:f>
+              <c:f>('combined sedimentary pteropods'!$Y$3,'combined sedimentary pteropods'!$Y$5)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1061,7 +1064,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>('combined sedimentary pteropods'!$AB$3,'combined sedimentary pteropods'!$AB$5)</c:f>
+              <c:f>('combined sedimentary pteropods'!$AC$3,'combined sedimentary pteropods'!$AC$5)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1111,7 +1114,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>('workup for cleaning types'!$X$7,'workup for cleaning types'!$X$8)</c:f>
+              <c:f>('workup for cleaning types'!$Y$7,'workup for cleaning types'!$Y$8)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1126,7 +1129,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>('workup for cleaning types'!$Y$7,'workup for cleaning types'!$Y$8)</c:f>
+              <c:f>('workup for cleaning types'!$Z$7,'workup for cleaning types'!$Z$8)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1176,7 +1179,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>('workup for cleaning types'!$X$9,'workup for cleaning types'!$X$10,'workup for cleaning types'!$X$11)</c:f>
+              <c:f>('workup for cleaning types'!$Y$9,'workup for cleaning types'!$Y$10,'workup for cleaning types'!$Y$11)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1194,7 +1197,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>('workup for cleaning types'!$Y$9,'workup for cleaning types'!$Y$10,'workup for cleaning types'!$Y$11)</c:f>
+              <c:f>('workup for cleaning types'!$Z$9,'workup for cleaning types'!$Z$10,'workup for cleaning types'!$Z$11)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1247,7 +1250,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>('workup for cleaning types'!$X$12,'workup for cleaning types'!$X$14)</c:f>
+              <c:f>('workup for cleaning types'!$Y$12,'workup for cleaning types'!$Y$14)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1262,7 +1265,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>('workup for cleaning types'!$Y$12,'workup for cleaning types'!$Y$14)</c:f>
+              <c:f>('workup for cleaning types'!$Z$12,'workup for cleaning types'!$Z$14)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -3439,13 +3442,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>22</xdr:col>
+      <xdr:col>23</xdr:col>
       <xdr:colOff>792480</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>20320</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
+      <xdr:col>33</xdr:col>
       <xdr:colOff>375920</xdr:colOff>
       <xdr:row>32</xdr:row>
       <xdr:rowOff>91440</xdr:rowOff>
@@ -3480,13 +3483,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>22</xdr:col>
+      <xdr:col>23</xdr:col>
       <xdr:colOff>779780</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>34</xdr:col>
+      <xdr:col>35</xdr:col>
       <xdr:colOff>215900</xdr:colOff>
       <xdr:row>44</xdr:row>
       <xdr:rowOff>177800</xdr:rowOff>
@@ -3518,13 +3521,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>34</xdr:col>
+      <xdr:col>35</xdr:col>
       <xdr:colOff>793750</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>44</xdr:col>
+      <xdr:col>45</xdr:col>
       <xdr:colOff>596900</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
@@ -3563,7 +3566,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="30041850" y="609600"/>
+              <a:off x="30968950" y="609600"/>
               <a:ext cx="8058150" cy="5702300"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -3914,41 +3917,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E48682E5-9042-AA48-86DE-B01B9E181CE6}">
-  <dimension ref="A1:AC18"/>
+  <dimension ref="A1:AD18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="13" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="17.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" customWidth="1"/>
+    <col min="22" max="22" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>59</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>46</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>47</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>56</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>64</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>57</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AD1" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3962,79 +3966,82 @@
         <v>19</v>
       </c>
       <c r="E2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" t="s">
         <v>20</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>21</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>22</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>23</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>24</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>25</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>26</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>27</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>31</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>28</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>32</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>29</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>28</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>30</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>28</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>53</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>52</v>
       </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
         <v>54</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>55</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>65</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AA2" t="s">
         <v>66</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AB2" t="s">
         <v>61</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AC2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -4047,87 +4054,90 @@
       <c r="D3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+      <c r="F3">
         <v>2.4240384752474555</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>11.994102980491613</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>468.38955954380759</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>17.210719873136657</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>9.0461226093249802</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>175.65853023117276</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>556.80649953290072</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>513.90317393468467</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>0.61011236389919465</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>9.659858120147833E-3</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>0.53802649664980173</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>8.7594674974638773E-3</v>
       </c>
-      <c r="Q3">
+      <c r="R3">
         <v>0.88457133958835987</v>
       </c>
-      <c r="R3">
+      <c r="S3">
         <v>1.398907150507946E-2</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <v>0.78005765337052135</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>2.5140929474624894E-3</v>
       </c>
-      <c r="U3">
-        <f>(((Q3/(2.22*10^12))/(6.22*10^-3))/234.04095)*10^9</f>
+      <c r="V3">
+        <f>(((R3/(2.22*10^12))/(6.22*10^-3))/234.04095)*10^9</f>
         <v>2.7371440408043132E-4</v>
       </c>
-      <c r="V3">
-        <f>(((S3/(2.22*10^12))/(3.36*10^-7))/238.05079)*10^9</f>
+      <c r="W3">
+        <f>(((T3/(2.22*10^12))/(3.36*10^-7))/238.05079)*10^9</f>
         <v>4.3930366175877529</v>
       </c>
-      <c r="W3">
-        <f t="shared" ref="W3:W12" si="0">U3*100.0869</f>
+      <c r="X3">
+        <f t="shared" ref="X3:X12" si="0">V3*100.0869</f>
         <v>2.7395226189757722E-2</v>
       </c>
-      <c r="X3">
-        <f t="shared" ref="X3:X12" si="1">V3*100.0869</f>
+      <c r="Y3">
+        <f t="shared" ref="Y3:Y12" si="1">W3*100.0869</f>
         <v>439.68541664084364</v>
       </c>
-      <c r="Y3">
-        <f>W3/0.0055</f>
+      <c r="Z3">
+        <f>X3/0.0055</f>
         <v>4.9809502163195862</v>
       </c>
-      <c r="Z3">
-        <f>X3/99.28</f>
+      <c r="AA3">
+        <f>Y3/99.28</f>
         <v>4.4287411023453229</v>
       </c>
-      <c r="AA3">
-        <f>Y3/Z3</f>
+      <c r="AB3">
+        <f>Z3/AA3</f>
         <v>1.1246876033647193</v>
       </c>
-      <c r="AB3">
+      <c r="AC3">
         <v>468.38955954380799</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -4140,90 +4150,93 @@
       <c r="D4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+      <c r="F4">
         <v>2.3029585788126603</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>12.848314913862716</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>447.94133990479213</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>17.48493818558244</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>8.1723364792775737</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>174.43419391518393</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>588.74721751902257</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>627.11718748768214</v>
       </c>
-      <c r="M4" s="6">
+      <c r="N4" s="6">
         <v>0.32184415565315633</v>
       </c>
-      <c r="N4" s="6">
+      <c r="O4" s="6">
         <v>1.9759427368043841E-2</v>
       </c>
-      <c r="O4" s="6">
+      <c r="P4" s="6">
         <v>0.31655296802723609</v>
       </c>
-      <c r="P4" s="6">
+      <c r="Q4" s="6">
         <v>1.9631098958537853E-2</v>
       </c>
-      <c r="Q4" s="6">
+      <c r="R4" s="6">
         <v>1.5182451480385759</v>
       </c>
-      <c r="R4" s="6">
+      <c r="S4" s="6">
         <v>2.7959826102772593E-2</v>
       </c>
-      <c r="S4" s="6">
+      <c r="T4" s="6">
         <v>1.4932848689739704</v>
       </c>
-      <c r="T4" s="6">
+      <c r="U4" s="6">
         <v>1.7982019455003682E-2</v>
       </c>
-      <c r="U4" s="6">
-        <f t="shared" ref="U4:U14" si="2">(((Q4/(2.22*10^12))/(6.22*10^-3))/234.04095)*10^9</f>
+      <c r="V4" s="6">
+        <f t="shared" ref="V4:V14" si="2">(((R4/(2.22*10^12))/(6.22*10^-3))/234.04095)*10^9</f>
         <v>4.6979316121271883E-4</v>
       </c>
-      <c r="V4" s="6">
-        <f t="shared" ref="V4:V14" si="3">(((S4/(2.22*10^12))/(3.36*10^-7))/238.05079)*10^9</f>
+      <c r="W4" s="6">
+        <f t="shared" ref="W4:W14" si="3">(((T4/(2.22*10^12))/(3.36*10^-7))/238.05079)*10^9</f>
         <v>8.4097054641375415</v>
       </c>
-      <c r="W4" s="6">
-        <f>U4*100.0869</f>
+      <c r="X4" s="6">
+        <f>V4*100.0869</f>
         <v>4.7020141146981269E-2</v>
       </c>
-      <c r="X4" s="6">
+      <c r="Y4" s="6">
         <f t="shared" si="1"/>
         <v>841.70134981858769</v>
       </c>
-      <c r="Y4">
-        <f t="shared" ref="Y4:Y14" si="4">W4/0.0055</f>
+      <c r="Z4">
+        <f t="shared" ref="Z4:Z14" si="4">X4/0.0055</f>
         <v>8.5491165721784128</v>
       </c>
-      <c r="Z4">
-        <f t="shared" ref="Z4:Z14" si="5">X4/99.28</f>
+      <c r="AA4">
+        <f t="shared" ref="AA4:AA14" si="5">Y4/99.28</f>
         <v>8.4780554977698195</v>
       </c>
-      <c r="AA4">
-        <f t="shared" ref="AA4:AA14" si="6">Y4/Z4</f>
+      <c r="AB4">
+        <f t="shared" ref="AB4:AB14" si="6">Z4/AA4</f>
         <v>1.0083817656569112</v>
       </c>
-      <c r="AB4" s="6">
+      <c r="AC4" s="6">
         <v>447.94133990479213</v>
       </c>
-      <c r="AC4" s="6" t="s">
+      <c r="AD4" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -4236,87 +4249,90 @@
       <c r="D5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="3">
+        <v>1</v>
+      </c>
+      <c r="F5">
         <v>2.345928293878571</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>12.4210935332361</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>449.29715930327058</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>17.329182493403763</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>9.0241428147331195</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>165.6397343820345</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>521.81682436992435</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>548.66957616592072</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>0.6113403454519396</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>1.1098193331586362E-2</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>0.52224101843495452</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>9.7325829515663188E-3</v>
       </c>
-      <c r="Q5">
+      <c r="R5">
         <v>0.92570447024607938</v>
       </c>
-      <c r="R5">
+      <c r="S5">
         <v>1.5014527363940051E-2</v>
       </c>
-      <c r="S5">
+      <c r="T5">
         <v>0.79078838638355209</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <v>2.8617150934306121E-3</v>
       </c>
-      <c r="U5">
+      <c r="V5">
         <f t="shared" si="2"/>
         <v>2.8644229819373086E-4</v>
       </c>
-      <c r="V5">
+      <c r="W5">
         <f t="shared" si="3"/>
         <v>4.4534686931607759</v>
       </c>
-      <c r="W5">
+      <c r="X5">
         <f t="shared" si="0"/>
         <v>2.8669121655086123E-2</v>
       </c>
-      <c r="X5">
+      <c r="Y5">
         <f t="shared" si="1"/>
         <v>445.73387574551327</v>
       </c>
-      <c r="Y5">
+      <c r="Z5">
         <f t="shared" si="4"/>
         <v>5.2125675736520227</v>
       </c>
-      <c r="Z5">
+      <c r="AA5">
         <f t="shared" si="5"/>
         <v>4.4896643407082317</v>
       </c>
-      <c r="AA5">
+      <c r="AB5">
         <f t="shared" si="6"/>
         <v>1.161014984213665</v>
       </c>
-      <c r="AB5">
+      <c r="AC5">
         <v>449.29715930327058</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -4329,90 +4345,93 @@
       <c r="D6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="4">
+        <v>2</v>
+      </c>
+      <c r="F6">
         <v>1.5770705354627657</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>6.7189407304641602</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>302.79267025152586</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>18.657383483251486</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>3.1512495171605153</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>48.952169951362642</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>174.51428541350577</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>219.93697957266215</v>
       </c>
-      <c r="M6" s="6">
+      <c r="N6" s="6">
         <v>0.11545108744532581</v>
       </c>
-      <c r="N6" s="6">
+      <c r="O6" s="6">
         <v>3.5591381972850744E-3</v>
       </c>
-      <c r="O6" s="6">
+      <c r="P6" s="6">
         <v>0.11362729477299752</v>
       </c>
-      <c r="P6" s="6">
+      <c r="Q6" s="6">
         <v>3.6524543911072216E-3</v>
       </c>
-      <c r="Q6" s="6">
+      <c r="R6" s="6">
         <v>1.4129186566526521</v>
       </c>
-      <c r="R6" s="6">
+      <c r="S6" s="6">
         <v>2.513698068564111E-2</v>
       </c>
-      <c r="S6" s="6">
+      <c r="T6" s="6">
         <v>1.3905986356842974</v>
       </c>
-      <c r="T6" s="6">
+      <c r="U6" s="6">
         <v>1.8112674916098581E-2</v>
       </c>
-      <c r="U6" s="6">
+      <c r="V6" s="6">
         <f t="shared" si="2"/>
         <v>4.3720180703545519E-4</v>
       </c>
-      <c r="V6" s="6">
+      <c r="W6" s="6">
         <f t="shared" si="3"/>
         <v>7.8314092561399251</v>
       </c>
-      <c r="W6" s="6">
+      <c r="X6" s="6">
         <f t="shared" si="0"/>
         <v>4.37581735405769E-2</v>
       </c>
-      <c r="X6" s="6">
+      <c r="Y6" s="6">
         <f t="shared" si="1"/>
         <v>783.82147507835111</v>
       </c>
-      <c r="Y6">
+      <c r="Z6">
         <f t="shared" si="4"/>
         <v>7.9560315528321643</v>
       </c>
-      <c r="Z6">
+      <c r="AA6">
         <f t="shared" si="5"/>
         <v>7.895059176856881</v>
       </c>
-      <c r="AA6">
+      <c r="AB6">
         <f t="shared" si="6"/>
         <v>1.0077228523066697</v>
       </c>
-      <c r="AB6" s="6">
+      <c r="AC6" s="6">
         <v>302.79267025152586</v>
       </c>
-      <c r="AC6" s="6" t="s">
+      <c r="AD6" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -4425,87 +4444,90 @@
       <c r="D7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="4">
+        <v>2</v>
+      </c>
+      <c r="F7">
         <v>1.5979015509006576</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>7.0066786694995518</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>308.31198972930645</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>18.821290469293292</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>3.4112927201749854</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>47.295715951994339</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>167.46871571763438</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>156.34316228209411</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>0.28793120032151515</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>8.8994850722590793E-3</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>0.25014198454203973</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>8.3584493007054679E-3</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>0.61502865442679866</v>
       </c>
-      <c r="R7">
+      <c r="S7">
         <v>1.5491320210685619E-2</v>
       </c>
-      <c r="S7">
+      <c r="T7">
         <v>0.53430989068482693</v>
       </c>
-      <c r="T7">
+      <c r="U7">
         <v>1.5663645505708649E-3</v>
       </c>
-      <c r="U7">
+      <c r="V7">
         <f t="shared" si="2"/>
         <v>1.9030935562207982E-4</v>
       </c>
-      <c r="V7">
+      <c r="W7">
         <f t="shared" si="3"/>
         <v>3.0090633747078073</v>
       </c>
-      <c r="W7">
+      <c r="X7">
         <f t="shared" si="0"/>
         <v>1.904747344521154E-2</v>
       </c>
-      <c r="X7">
+      <c r="Y7">
         <f t="shared" si="1"/>
         <v>301.16782507804282</v>
       </c>
-      <c r="Y7">
+      <c r="Z7">
         <f t="shared" si="4"/>
         <v>3.4631769900384621</v>
       </c>
-      <c r="Z7">
+      <c r="AA7">
         <f t="shared" si="5"/>
         <v>3.0335195918416882</v>
       </c>
-      <c r="AA7">
+      <c r="AB7">
         <f t="shared" si="6"/>
         <v>1.1416365990687152</v>
       </c>
-      <c r="AB7">
+      <c r="AC7">
         <v>308.31198972930645</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -4518,87 +4540,90 @@
       <c r="D8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="4">
+        <v>2</v>
+      </c>
+      <c r="F8">
         <v>1.6682384240136723</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>7.2962224303392018</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>320.71440975593009</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>18.326195021745924</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>3.5690384469412031</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>44.414757823823244</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>157.62759062691416</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <v>141.92032139848197</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>0.26745036769803937</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>1.1832331707506256E-2</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>0.23195391778314434</v>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <v>1.0783570590813113E-2</v>
       </c>
-      <c r="Q8">
+      <c r="R8">
         <v>0.64142579192172633</v>
       </c>
-      <c r="R8">
+      <c r="S8">
         <v>1.4868572449519658E-2</v>
       </c>
-      <c r="S8">
+      <c r="T8">
         <v>0.55629471248803608</v>
       </c>
-      <c r="T8">
+      <c r="U8">
         <v>2.3661545080180995E-3</v>
       </c>
-      <c r="U8">
+      <c r="V8">
         <f t="shared" si="2"/>
         <v>1.9847746647475074E-4</v>
       </c>
-      <c r="V8">
+      <c r="W8">
         <f t="shared" si="3"/>
         <v>3.1328748991449182</v>
       </c>
-      <c r="W8">
+      <c r="X8">
         <f t="shared" si="0"/>
         <v>1.9864994339311732E-2</v>
       </c>
-      <c r="X8">
+      <c r="Y8">
         <f t="shared" si="1"/>
         <v>313.55973674322752</v>
       </c>
-      <c r="Y8">
+      <c r="Z8">
         <f t="shared" si="4"/>
         <v>3.6118171526021334</v>
       </c>
-      <c r="Z8">
+      <c r="AA8">
         <f t="shared" si="5"/>
         <v>3.1583373966884318</v>
       </c>
-      <c r="AA8">
+      <c r="AB8">
         <f t="shared" si="6"/>
         <v>1.1435817960390118</v>
       </c>
-      <c r="AB8">
+      <c r="AC8">
         <v>320.71440975593009</v>
       </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -4611,87 +4636,90 @@
       <c r="D9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="4">
+        <v>3</v>
+      </c>
+      <c r="F9">
         <v>1.3415621166647502</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>5.7020981777185344</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>223.36742932630972</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>18.673299261589669</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>1.1983217414583234</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>15.484944635332528</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>25.883426323940235</v>
       </c>
-      <c r="L9">
+      <c r="M9">
         <v>72.380084089451174</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>0.11467667624357794</v>
       </c>
-      <c r="N9">
+      <c r="O9">
         <v>4.7935019894853655E-3</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>0.10000325369432765</v>
       </c>
-      <c r="P9">
+      <c r="Q9">
         <v>4.7882548765769859E-3</v>
       </c>
-      <c r="Q9">
+      <c r="R9">
         <v>0.43617366290414139</v>
       </c>
-      <c r="R9">
+      <c r="S9">
         <v>1.0863870018925463E-2</v>
       </c>
-      <c r="S9">
+      <c r="T9">
         <v>0.38036318190404228</v>
       </c>
-      <c r="T9">
+      <c r="U9">
         <v>1.4264766471405556E-3</v>
       </c>
-      <c r="U9">
+      <c r="V9">
         <f t="shared" si="2"/>
         <v>1.3496595342207604E-4</v>
       </c>
-      <c r="V9">
+      <c r="W9">
         <f t="shared" si="3"/>
         <v>2.1420844714063221</v>
       </c>
-      <c r="W9">
+      <c r="X9">
         <f t="shared" si="0"/>
         <v>1.3508323883559981E-2</v>
       </c>
-      <c r="X9">
+      <c r="Y9">
         <f t="shared" si="1"/>
         <v>214.39459428119741</v>
       </c>
-      <c r="Y9">
+      <c r="Z9">
         <f t="shared" si="4"/>
         <v>2.4560588879199967</v>
       </c>
-      <c r="Z9">
+      <c r="AA9">
         <f t="shared" si="5"/>
         <v>2.1594943017848247</v>
       </c>
-      <c r="AA9">
+      <c r="AB9">
         <f t="shared" si="6"/>
         <v>1.1373305712777575</v>
       </c>
-      <c r="AB9">
+      <c r="AC9">
         <v>223.36742932630972</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -4704,87 +4732,90 @@
       <c r="D10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="4">
+        <v>3</v>
+      </c>
+      <c r="F10">
         <v>1.5575845128239232</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>5.9421197851468381</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>236.96242951649464</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>29.761961607080888</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>1.4098955149865431</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>15.630759401881026</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>25.786920422638271</v>
       </c>
-      <c r="L10">
+      <c r="M10">
         <v>53.637733087144142</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <v>0.10715733028928495</v>
       </c>
-      <c r="N10">
+      <c r="O10">
         <v>4.8073149006271779E-3</v>
       </c>
-      <c r="O10">
+      <c r="P10">
         <v>9.3118538656026081E-2</v>
       </c>
-      <c r="P10">
+      <c r="Q10">
         <v>4.3796363697899705E-3</v>
       </c>
-      <c r="Q10">
+      <c r="R10">
         <v>0.4550012663976748</v>
       </c>
-      <c r="R10">
+      <c r="S10">
         <v>6.6397480068390528E-3</v>
       </c>
-      <c r="S10">
+      <c r="T10">
         <v>0.39539108429831171</v>
       </c>
-      <c r="T10">
+      <c r="U10">
         <v>1.3950254070308659E-3</v>
       </c>
-      <c r="U10">
+      <c r="V10">
         <f t="shared" si="2"/>
         <v>1.4079181058006772E-4</v>
       </c>
-      <c r="V10">
+      <c r="W10">
         <f t="shared" si="3"/>
         <v>2.2267168382811358</v>
       </c>
-      <c r="W10">
+      <c r="X10">
         <f t="shared" si="0"/>
         <v>1.409141586634618E-2</v>
       </c>
-      <c r="X10">
+      <c r="Y10">
         <f t="shared" si="1"/>
         <v>222.86518552136022</v>
       </c>
-      <c r="Y10">
+      <c r="Z10">
         <f t="shared" si="4"/>
         <v>2.5620756120629418</v>
       </c>
-      <c r="Z10">
+      <c r="AA10">
         <f t="shared" si="5"/>
         <v>2.244814519755844</v>
       </c>
-      <c r="AA10">
+      <c r="AB10">
         <f t="shared" si="6"/>
         <v>1.1413306487083861</v>
       </c>
-      <c r="AB10">
+      <c r="AC10">
         <v>236.96242951649464</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -4797,87 +4828,90 @@
       <c r="D11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="4">
+        <v>3</v>
+      </c>
+      <c r="F11">
         <v>1.4277933288311244</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <v>6.3871622724129553</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>247.06680639675164</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>18.790528988644279</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>0.92571492034021241</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>15.710662717164421</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>30.053589541503872</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <v>59.876917988874879</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>0.10381470441637841</v>
       </c>
-      <c r="N11">
+      <c r="O11">
         <v>3.6417684292928323E-3</v>
       </c>
-      <c r="O11">
+      <c r="P11">
         <v>9.0593462356721971E-2</v>
       </c>
-      <c r="P11">
+      <c r="Q11">
         <v>3.4922246772751049E-3</v>
       </c>
-      <c r="Q11">
+      <c r="R11">
         <v>0.44557097161871734</v>
       </c>
-      <c r="R11">
+      <c r="S11">
         <v>8.0681617295171419E-3</v>
       </c>
-      <c r="S11">
+      <c r="T11">
         <v>0.38882562226146411</v>
       </c>
-      <c r="T11">
+      <c r="U11">
         <v>1.536652745364092E-3</v>
       </c>
-      <c r="U11">
+      <c r="V11">
         <f t="shared" si="2"/>
         <v>1.3787377853425632E-4</v>
       </c>
-      <c r="V11">
+      <c r="W11">
         <f t="shared" si="3"/>
         <v>2.1897422441410357</v>
       </c>
-      <c r="W11">
+      <c r="X11">
         <f t="shared" si="0"/>
         <v>1.379935908478026E-2</v>
       </c>
-      <c r="X11">
+      <c r="Y11">
         <f t="shared" si="1"/>
         <v>219.16451301511941</v>
       </c>
-      <c r="Y11">
+      <c r="Z11">
         <f t="shared" si="4"/>
         <v>2.5089743790509567</v>
       </c>
-      <c r="Z11">
+      <c r="AA11">
         <f t="shared" si="5"/>
         <v>2.2075394139315008</v>
       </c>
-      <c r="AA11">
+      <c r="AB11">
         <f t="shared" si="6"/>
         <v>1.1365479425722314</v>
       </c>
-      <c r="AB11">
+      <c r="AC11">
         <v>247.06680639675164</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -4890,87 +4924,90 @@
       <c r="D12" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="4">
+        <v>4</v>
+      </c>
+      <c r="F12">
         <v>1.3244922852859213</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>6.4856878848228394</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>218.43171399770733</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>19.685248179403228</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>0.96641509427694361</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>15.895692464599502</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>17.47462352076996</v>
       </c>
-      <c r="L12">
+      <c r="M12">
         <v>45.282253824305165</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>9.6602107312809368E-2</v>
       </c>
-      <c r="N12">
+      <c r="O12">
         <v>3.377014314032404E-3</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <v>8.3287011253041374E-2</v>
       </c>
-      <c r="P12">
+      <c r="Q12">
         <v>3.0884230327830179E-3</v>
       </c>
-      <c r="Q12">
+      <c r="R12">
         <v>0.43924003179876875</v>
       </c>
-      <c r="R12">
+      <c r="S12">
         <v>5.9434640668399917E-3</v>
       </c>
-      <c r="S12">
+      <c r="T12">
         <v>0.37869763392169214</v>
       </c>
-      <c r="T12">
+      <c r="U12">
         <v>1.0169233741542834E-3</v>
       </c>
-      <c r="U12">
+      <c r="V12">
         <f t="shared" si="2"/>
         <v>1.3591478512973038E-4</v>
       </c>
-      <c r="V12">
+      <c r="W12">
         <f t="shared" si="3"/>
         <v>2.1327046348734728</v>
       </c>
-      <c r="W12">
+      <c r="X12">
         <f t="shared" si="0"/>
         <v>1.3603289507800811E-2</v>
       </c>
-      <c r="X12">
+      <c r="Y12">
         <f t="shared" si="1"/>
         <v>213.45579552011779</v>
       </c>
-      <c r="Y12">
+      <c r="Z12">
         <f t="shared" si="4"/>
         <v>2.4733253650546931</v>
       </c>
-      <c r="Z12">
+      <c r="AA12">
         <f t="shared" si="5"/>
         <v>2.1500382304604932</v>
       </c>
-      <c r="AA12">
+      <c r="AB12">
         <f t="shared" si="6"/>
         <v>1.150363435409685</v>
       </c>
-      <c r="AB12">
+      <c r="AC12">
         <v>218.43171399770733</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -4983,38 +5020,41 @@
       <c r="D13" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="4">
+        <v>4</v>
+      </c>
+      <c r="F13">
         <v>1.3081440292087358</v>
       </c>
-      <c r="F13">
+      <c r="G13">
         <v>6.0094659185272432</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>221.35630060801955</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>19.410276393833488</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>0.79350979357986651</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>15.74809501785283</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>23.308749817709145</v>
       </c>
-      <c r="L13">
+      <c r="M13">
         <v>62.512748584023385</v>
       </c>
-      <c r="AB13">
+      <c r="AC13">
         <v>221.35630060801955</v>
       </c>
-      <c r="AC13" s="7" t="s">
+      <c r="AD13" s="7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -5027,93 +5067,96 @@
       <c r="D14" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="4">
+        <v>4</v>
+      </c>
+      <c r="F14">
         <v>1.4717601344048605</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>6.7204925698794984</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>230.31890204975423</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>18.902391052529889</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>3.0758591947397695</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>14.818881820090528</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>19.593911628595208</v>
       </c>
-      <c r="L14">
+      <c r="M14">
         <v>46.069786166823988</v>
       </c>
-      <c r="M14">
+      <c r="N14">
         <v>0.10552467529276917</v>
       </c>
-      <c r="N14">
+      <c r="O14">
         <v>6.1133180135337362E-3</v>
       </c>
-      <c r="O14">
+      <c r="P14">
         <v>9.2195698250787522E-2</v>
       </c>
-      <c r="P14">
+      <c r="Q14">
         <v>5.6213880343485654E-3</v>
       </c>
-      <c r="Q14">
+      <c r="R14">
         <v>0.45817645066355467</v>
       </c>
-      <c r="R14">
+      <c r="S14">
         <v>7.7892390829879419E-3</v>
       </c>
-      <c r="S14">
+      <c r="T14">
         <v>0.40030350885986998</v>
       </c>
-      <c r="T14">
+      <c r="U14">
         <v>1.2679457836137552E-3</v>
       </c>
-      <c r="U14">
+      <c r="V14">
         <f t="shared" si="2"/>
         <v>1.4177431321189086E-4</v>
       </c>
-      <c r="V14">
+      <c r="W14">
         <f t="shared" si="3"/>
         <v>2.2543820510853649</v>
       </c>
-      <c r="W14">
-        <f>U14*100.0869</f>
-        <v>1.41897515090072E-2</v>
-      </c>
       <c r="X14">
         <f>V14*100.0869</f>
+        <v>1.41897515090072E-2</v>
+      </c>
+      <c r="Y14">
+        <f>W14*100.0869</f>
         <v>225.63411090877582</v>
       </c>
-      <c r="Y14">
+      <c r="Z14">
         <f t="shared" si="4"/>
         <v>2.5799548198194908</v>
       </c>
-      <c r="Z14">
+      <c r="AA14">
         <f t="shared" si="5"/>
         <v>2.2727045820787248</v>
       </c>
-      <c r="AA14">
+      <c r="AB14">
         <f t="shared" si="6"/>
         <v>1.135191454341919</v>
       </c>
-      <c r="AB14">
+      <c r="AC14">
         <v>230.31890204975423</v>
       </c>
     </row>
-    <row r="18" spans="17:22" x14ac:dyDescent="0.2">
-      <c r="Q18" s="6"/>
+    <row r="18" spans="18:23" x14ac:dyDescent="0.2">
       <c r="R18" s="6"/>
       <c r="S18" s="6"/>
       <c r="T18" s="6"/>
       <c r="U18" s="6"/>
       <c r="V18" s="6"/>
+      <c r="W18" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5333,17 +5376,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96C6F836-0A49-3E43-8E37-6BA61BFB5B6F}">
-  <dimension ref="A1:Z18"/>
+  <dimension ref="A1:AA18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="17.83203125" customWidth="1"/>
+    <col min="2" max="3" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -5354,90 +5399,93 @@
         <v>18</v>
       </c>
       <c r="D1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>46</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>47</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>56</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>57</v>
       </c>
-      <c r="Z1" s="5" t="s">
+      <c r="AA1" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="E2" t="s">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="F2" t="s">
         <v>20</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>21</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>22</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>23</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>24</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>25</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>26</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>27</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>31</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>28</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>32</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>29</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>28</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>30</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>28</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>53</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>52</v>
       </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
         <v>54</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>55</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -5447,78 +5495,81 @@
       <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>2.4240384752474555</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>11.994102980491613</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>468.38955954380759</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>17.210719873136657</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>9.0461226093249802</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>175.65853023117276</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>556.80649953290072</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>513.90317393468467</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>0.61011236389919465</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>9.659858120147833E-3</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>0.53802649664980173</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>8.7594674974638773E-3</v>
       </c>
-      <c r="Q3">
+      <c r="R3">
         <v>0.88457133958835987</v>
       </c>
-      <c r="R3">
+      <c r="S3">
         <v>1.398907150507946E-2</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <v>0.78005765337052135</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>2.5140929474624894E-3</v>
       </c>
-      <c r="U3">
-        <f>(((Q3/(2.22*10^12))/(6.22*10^-3))/234.04095)*10^9</f>
+      <c r="V3">
+        <f>(((R3/(2.22*10^12))/(6.22*10^-3))/234.04095)*10^9</f>
         <v>2.7371440408043132E-4</v>
       </c>
-      <c r="V3">
-        <f>(((S3/(2.22*10^12))/(3.36*10^-7))/238.05079)*10^9</f>
+      <c r="W3">
+        <f>(((T3/(2.22*10^12))/(3.36*10^-7))/238.05079)*10^9</f>
         <v>4.3930366175877529</v>
       </c>
-      <c r="W3">
-        <f t="shared" ref="W3:W12" si="0">U3*100.0869</f>
+      <c r="X3">
+        <f t="shared" ref="X3:X12" si="0">V3*100.0869</f>
         <v>2.7395226189757722E-2</v>
       </c>
-      <c r="X3">
-        <f t="shared" ref="X3:X12" si="1">V3*100.0869</f>
+      <c r="Y3">
+        <f t="shared" ref="Y3:Y12" si="1">W3*100.0869</f>
         <v>439.68541664084364</v>
       </c>
-      <c r="Y3">
+      <c r="Z3">
         <v>468.38955954380799</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -5528,81 +5579,84 @@
       <c r="C4" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>2.3029585788126603</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>12.848314913862716</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>447.94133990479213</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>17.48493818558244</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>8.1723364792775737</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>174.43419391518393</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>588.74721751902257</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>627.11718748768214</v>
       </c>
-      <c r="M4" s="6">
+      <c r="N4" s="6">
         <v>0.32184415565315633</v>
       </c>
-      <c r="N4" s="6">
+      <c r="O4" s="6">
         <v>1.9759427368043841E-2</v>
       </c>
-      <c r="O4" s="6">
+      <c r="P4" s="6">
         <v>0.31655296802723609</v>
       </c>
-      <c r="P4" s="6">
+      <c r="Q4" s="6">
         <v>1.9631098958537853E-2</v>
       </c>
-      <c r="Q4" s="6">
+      <c r="R4" s="6">
         <v>1.5182451480385759</v>
       </c>
-      <c r="R4" s="6">
+      <c r="S4" s="6">
         <v>2.7959826102772593E-2</v>
       </c>
-      <c r="S4" s="6">
+      <c r="T4" s="6">
         <v>1.4932848689739704</v>
       </c>
-      <c r="T4" s="6">
+      <c r="U4" s="6">
         <v>1.7982019455003682E-2</v>
       </c>
-      <c r="U4" s="6">
-        <f t="shared" ref="U4:U14" si="2">(((Q4/(2.22*10^12))/(6.22*10^-3))/234.04095)*10^9</f>
+      <c r="V4" s="6">
+        <f t="shared" ref="V4:V14" si="2">(((R4/(2.22*10^12))/(6.22*10^-3))/234.04095)*10^9</f>
         <v>4.6979316121271883E-4</v>
       </c>
-      <c r="V4" s="6">
-        <f t="shared" ref="V4:V14" si="3">(((S4/(2.22*10^12))/(3.36*10^-7))/238.05079)*10^9</f>
+      <c r="W4" s="6">
+        <f t="shared" ref="W4:W14" si="3">(((T4/(2.22*10^12))/(3.36*10^-7))/238.05079)*10^9</f>
         <v>8.4097054641375415</v>
       </c>
-      <c r="W4" s="6">
+      <c r="X4" s="6">
         <f t="shared" si="0"/>
         <v>4.7020141146981269E-2</v>
       </c>
-      <c r="X4" s="6">
+      <c r="Y4" s="6">
         <f t="shared" si="1"/>
         <v>841.70134981858769</v>
       </c>
-      <c r="Y4" s="6">
+      <c r="Z4" s="6">
         <v>447.94133990479213</v>
       </c>
-      <c r="Z4" s="6" t="s">
+      <c r="AA4" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -5612,78 +5666,81 @@
       <c r="C5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>2.345928293878571</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>12.4210935332361</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>449.29715930327058</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>17.329182493403763</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>9.0241428147331195</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>165.6397343820345</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>521.81682436992435</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>548.66957616592072</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>0.6113403454519396</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>1.1098193331586362E-2</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>0.52224101843495452</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>9.7325829515663188E-3</v>
       </c>
-      <c r="Q5">
+      <c r="R5">
         <v>0.92570447024607938</v>
       </c>
-      <c r="R5">
+      <c r="S5">
         <v>1.5014527363940051E-2</v>
       </c>
-      <c r="S5">
+      <c r="T5">
         <v>0.79078838638355209</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <v>2.8617150934306121E-3</v>
       </c>
-      <c r="U5">
+      <c r="V5">
         <f t="shared" si="2"/>
         <v>2.8644229819373086E-4</v>
       </c>
-      <c r="V5">
+      <c r="W5">
         <f t="shared" si="3"/>
         <v>4.4534686931607759</v>
       </c>
-      <c r="W5">
+      <c r="X5">
         <f t="shared" si="0"/>
         <v>2.8669121655086123E-2</v>
       </c>
-      <c r="X5">
+      <c r="Y5">
         <f t="shared" si="1"/>
         <v>445.73387574551327</v>
       </c>
-      <c r="Y5">
+      <c r="Z5">
         <v>449.29715930327058</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -5693,81 +5750,84 @@
       <c r="C6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="2">
+        <v>2</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>1.5770705354627657</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>6.7189407304641602</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>302.79267025152586</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>18.657383483251486</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>3.1512495171605153</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>48.952169951362642</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>174.51428541350577</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>219.93697957266215</v>
       </c>
-      <c r="M6" s="6">
+      <c r="N6" s="6">
         <v>0.11545108744532581</v>
       </c>
-      <c r="N6" s="6">
+      <c r="O6" s="6">
         <v>3.5591381972850744E-3</v>
       </c>
-      <c r="O6" s="6">
+      <c r="P6" s="6">
         <v>0.11362729477299752</v>
       </c>
-      <c r="P6" s="6">
+      <c r="Q6" s="6">
         <v>3.6524543911072216E-3</v>
       </c>
-      <c r="Q6" s="6">
+      <c r="R6" s="6">
         <v>1.4129186566526521</v>
       </c>
-      <c r="R6" s="6">
+      <c r="S6" s="6">
         <v>2.513698068564111E-2</v>
       </c>
-      <c r="S6" s="6">
+      <c r="T6" s="6">
         <v>1.3905986356842974</v>
       </c>
-      <c r="T6" s="6">
+      <c r="U6" s="6">
         <v>1.8112674916098581E-2</v>
       </c>
-      <c r="U6" s="6">
+      <c r="V6" s="6">
         <f t="shared" si="2"/>
         <v>4.3720180703545519E-4</v>
       </c>
-      <c r="V6" s="6">
+      <c r="W6" s="6">
         <f t="shared" si="3"/>
         <v>7.8314092561399251</v>
       </c>
-      <c r="W6" s="6">
+      <c r="X6" s="6">
         <f t="shared" si="0"/>
         <v>4.37581735405769E-2</v>
       </c>
-      <c r="X6" s="6">
+      <c r="Y6" s="6">
         <f t="shared" si="1"/>
         <v>783.82147507835111</v>
       </c>
-      <c r="Y6" s="6">
+      <c r="Z6" s="6">
         <v>302.79267025152586</v>
       </c>
-      <c r="Z6" s="6" t="s">
+      <c r="AA6" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -5777,78 +5837,81 @@
       <c r="C7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="2">
+        <v>2</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>1.5979015509006576</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>7.0066786694995518</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>308.31198972930645</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>18.821290469293292</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>3.4112927201749854</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>47.295715951994339</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>167.46871571763438</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>156.34316228209411</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>0.28793120032151515</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>8.8994850722590793E-3</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>0.25014198454203973</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>8.3584493007054679E-3</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>0.61502865442679866</v>
       </c>
-      <c r="R7">
+      <c r="S7">
         <v>1.5491320210685619E-2</v>
       </c>
-      <c r="S7">
+      <c r="T7">
         <v>0.53430989068482693</v>
       </c>
-      <c r="T7">
+      <c r="U7">
         <v>1.5663645505708649E-3</v>
       </c>
-      <c r="U7">
+      <c r="V7">
         <f t="shared" si="2"/>
         <v>1.9030935562207982E-4</v>
       </c>
-      <c r="V7">
+      <c r="W7">
         <f t="shared" si="3"/>
         <v>3.0090633747078073</v>
       </c>
-      <c r="W7">
+      <c r="X7">
         <f t="shared" si="0"/>
         <v>1.904747344521154E-2</v>
       </c>
-      <c r="X7">
+      <c r="Y7">
         <f t="shared" si="1"/>
         <v>301.16782507804282</v>
       </c>
-      <c r="Y7">
+      <c r="Z7">
         <v>308.31198972930645</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -5858,78 +5921,81 @@
       <c r="C8" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="2">
+        <v>2</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>1.6682384240136723</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>7.2962224303392018</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>320.71440975593009</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>18.326195021745924</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>3.5690384469412031</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>44.414757823823244</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>157.62759062691416</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <v>141.92032139848197</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>0.26745036769803937</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>1.1832331707506256E-2</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>0.23195391778314434</v>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <v>1.0783570590813113E-2</v>
       </c>
-      <c r="Q8">
+      <c r="R8">
         <v>0.64142579192172633</v>
       </c>
-      <c r="R8">
+      <c r="S8">
         <v>1.4868572449519658E-2</v>
       </c>
-      <c r="S8">
+      <c r="T8">
         <v>0.55629471248803608</v>
       </c>
-      <c r="T8">
+      <c r="U8">
         <v>2.3661545080180995E-3</v>
       </c>
-      <c r="U8">
+      <c r="V8">
         <f t="shared" si="2"/>
         <v>1.9847746647475074E-4</v>
       </c>
-      <c r="V8">
+      <c r="W8">
         <f t="shared" si="3"/>
         <v>3.1328748991449182</v>
       </c>
-      <c r="W8">
+      <c r="X8">
         <f t="shared" si="0"/>
         <v>1.9864994339311732E-2</v>
       </c>
-      <c r="X8">
+      <c r="Y8">
         <f t="shared" si="1"/>
         <v>313.55973674322752</v>
       </c>
-      <c r="Y8">
+      <c r="Z8">
         <v>320.71440975593009</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -5939,78 +6005,81 @@
       <c r="C9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="2">
+        <v>3</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>1.3415621166647502</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>5.7020981777185344</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>223.36742932630972</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>18.673299261589669</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>1.1983217414583234</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>15.484944635332528</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>25.883426323940235</v>
       </c>
-      <c r="L9">
+      <c r="M9">
         <v>72.380084089451174</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>0.11467667624357794</v>
       </c>
-      <c r="N9">
+      <c r="O9">
         <v>4.7935019894853655E-3</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>0.10000325369432765</v>
       </c>
-      <c r="P9">
+      <c r="Q9">
         <v>4.7882548765769859E-3</v>
       </c>
-      <c r="Q9">
+      <c r="R9">
         <v>0.43617366290414139</v>
       </c>
-      <c r="R9">
+      <c r="S9">
         <v>1.0863870018925463E-2</v>
       </c>
-      <c r="S9">
+      <c r="T9">
         <v>0.38036318190404228</v>
       </c>
-      <c r="T9">
+      <c r="U9">
         <v>1.4264766471405556E-3</v>
       </c>
-      <c r="U9">
+      <c r="V9">
         <f t="shared" si="2"/>
         <v>1.3496595342207604E-4</v>
       </c>
-      <c r="V9">
+      <c r="W9">
         <f t="shared" si="3"/>
         <v>2.1420844714063221</v>
       </c>
-      <c r="W9">
+      <c r="X9">
         <f t="shared" si="0"/>
         <v>1.3508323883559981E-2</v>
       </c>
-      <c r="X9">
+      <c r="Y9">
         <f t="shared" si="1"/>
         <v>214.39459428119741</v>
       </c>
-      <c r="Y9">
+      <c r="Z9">
         <v>223.36742932630972</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -6020,78 +6089,81 @@
       <c r="C10" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="2">
+        <v>3</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>1.5575845128239232</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>5.9421197851468381</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>236.96242951649464</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>29.761961607080888</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>1.4098955149865431</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>15.630759401881026</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>25.786920422638271</v>
       </c>
-      <c r="L10">
+      <c r="M10">
         <v>53.637733087144142</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <v>0.10715733028928495</v>
       </c>
-      <c r="N10">
+      <c r="O10">
         <v>4.8073149006271779E-3</v>
       </c>
-      <c r="O10">
+      <c r="P10">
         <v>9.3118538656026081E-2</v>
       </c>
-      <c r="P10">
+      <c r="Q10">
         <v>4.3796363697899705E-3</v>
       </c>
-      <c r="Q10">
+      <c r="R10">
         <v>0.4550012663976748</v>
       </c>
-      <c r="R10">
+      <c r="S10">
         <v>6.6397480068390528E-3</v>
       </c>
-      <c r="S10">
+      <c r="T10">
         <v>0.39539108429831171</v>
       </c>
-      <c r="T10">
+      <c r="U10">
         <v>1.3950254070308659E-3</v>
       </c>
-      <c r="U10">
+      <c r="V10">
         <f t="shared" si="2"/>
         <v>1.4079181058006772E-4</v>
       </c>
-      <c r="V10">
+      <c r="W10">
         <f t="shared" si="3"/>
         <v>2.2267168382811358</v>
       </c>
-      <c r="W10">
+      <c r="X10">
         <f t="shared" si="0"/>
         <v>1.409141586634618E-2</v>
       </c>
-      <c r="X10">
+      <c r="Y10">
         <f t="shared" si="1"/>
         <v>222.86518552136022</v>
       </c>
-      <c r="Y10">
+      <c r="Z10">
         <v>236.96242951649464</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -6101,78 +6173,81 @@
       <c r="C11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="2">
+        <v>3</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>1.4277933288311244</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <v>6.3871622724129553</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>247.06680639675164</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>18.790528988644279</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>0.92571492034021241</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>15.710662717164421</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>30.053589541503872</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <v>59.876917988874879</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>0.10381470441637841</v>
       </c>
-      <c r="N11">
+      <c r="O11">
         <v>3.6417684292928323E-3</v>
       </c>
-      <c r="O11">
+      <c r="P11">
         <v>9.0593462356721971E-2</v>
       </c>
-      <c r="P11">
+      <c r="Q11">
         <v>3.4922246772751049E-3</v>
       </c>
-      <c r="Q11">
+      <c r="R11">
         <v>0.44557097161871734</v>
       </c>
-      <c r="R11">
+      <c r="S11">
         <v>8.0681617295171419E-3</v>
       </c>
-      <c r="S11">
+      <c r="T11">
         <v>0.38882562226146411</v>
       </c>
-      <c r="T11">
+      <c r="U11">
         <v>1.536652745364092E-3</v>
       </c>
-      <c r="U11">
+      <c r="V11">
         <f t="shared" si="2"/>
         <v>1.3787377853425632E-4</v>
       </c>
-      <c r="V11">
+      <c r="W11">
         <f t="shared" si="3"/>
         <v>2.1897422441410357</v>
       </c>
-      <c r="W11">
+      <c r="X11">
         <f t="shared" si="0"/>
         <v>1.379935908478026E-2</v>
       </c>
-      <c r="X11">
+      <c r="Y11">
         <f t="shared" si="1"/>
         <v>219.16451301511941</v>
       </c>
-      <c r="Y11">
+      <c r="Z11">
         <v>247.06680639675164</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -6182,78 +6257,81 @@
       <c r="C12" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="2">
+        <v>4</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>1.3244922852859213</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>6.4856878848228394</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>218.43171399770733</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>19.685248179403228</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>0.96641509427694361</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>15.895692464599502</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>17.47462352076996</v>
       </c>
-      <c r="L12">
+      <c r="M12">
         <v>45.282253824305165</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>9.6602107312809368E-2</v>
       </c>
-      <c r="N12">
+      <c r="O12">
         <v>3.377014314032404E-3</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <v>8.3287011253041374E-2</v>
       </c>
-      <c r="P12">
+      <c r="Q12">
         <v>3.0884230327830179E-3</v>
       </c>
-      <c r="Q12">
+      <c r="R12">
         <v>0.43924003179876875</v>
       </c>
-      <c r="R12">
+      <c r="S12">
         <v>5.9434640668399917E-3</v>
       </c>
-      <c r="S12">
+      <c r="T12">
         <v>0.37869763392169214</v>
       </c>
-      <c r="T12">
+      <c r="U12">
         <v>1.0169233741542834E-3</v>
       </c>
-      <c r="U12">
+      <c r="V12">
         <f t="shared" si="2"/>
         <v>1.3591478512973038E-4</v>
       </c>
-      <c r="V12">
+      <c r="W12">
         <f t="shared" si="3"/>
         <v>2.1327046348734728</v>
       </c>
-      <c r="W12">
+      <c r="X12">
         <f t="shared" si="0"/>
         <v>1.3603289507800811E-2</v>
       </c>
-      <c r="X12">
+      <c r="Y12">
         <f t="shared" si="1"/>
         <v>213.45579552011779</v>
       </c>
-      <c r="Y12">
+      <c r="Z12">
         <v>218.43171399770733</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -6263,41 +6341,44 @@
       <c r="C13" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="2">
+        <v>4</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <v>1.3081440292087358</v>
       </c>
-      <c r="F13">
+      <c r="G13">
         <v>6.0094659185272432</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>221.35630060801955</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>19.410276393833488</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>0.79350979357986651</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>15.74809501785283</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>23.308749817709145</v>
       </c>
-      <c r="L13">
+      <c r="M13">
         <v>62.512748584023385</v>
       </c>
-      <c r="Y13">
+      <c r="Z13">
         <v>221.35630060801955</v>
       </c>
-      <c r="Z13" s="7" t="s">
+      <c r="AA13" s="7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -6307,84 +6388,87 @@
       <c r="C14" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="2">
+        <v>4</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <v>1.4717601344048605</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>6.7204925698794984</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>230.31890204975423</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>18.902391052529889</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>3.0758591947397695</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>14.818881820090528</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>19.593911628595208</v>
       </c>
-      <c r="L14">
+      <c r="M14">
         <v>46.069786166823988</v>
       </c>
-      <c r="M14">
+      <c r="N14">
         <v>0.10552467529276917</v>
       </c>
-      <c r="N14">
+      <c r="O14">
         <v>6.1133180135337362E-3</v>
       </c>
-      <c r="O14">
+      <c r="P14">
         <v>9.2195698250787522E-2</v>
       </c>
-      <c r="P14">
+      <c r="Q14">
         <v>5.6213880343485654E-3</v>
       </c>
-      <c r="Q14">
+      <c r="R14">
         <v>0.45817645066355467</v>
       </c>
-      <c r="R14">
+      <c r="S14">
         <v>7.7892390829879419E-3</v>
       </c>
-      <c r="S14">
+      <c r="T14">
         <v>0.40030350885986998</v>
       </c>
-      <c r="T14">
+      <c r="U14">
         <v>1.2679457836137552E-3</v>
       </c>
-      <c r="U14">
+      <c r="V14">
         <f t="shared" si="2"/>
         <v>1.4177431321189086E-4</v>
       </c>
-      <c r="V14">
+      <c r="W14">
         <f t="shared" si="3"/>
         <v>2.2543820510853649</v>
       </c>
-      <c r="W14">
-        <f>U14*100.0869</f>
-        <v>1.41897515090072E-2</v>
-      </c>
       <c r="X14">
         <f>V14*100.0869</f>
+        <v>1.41897515090072E-2</v>
+      </c>
+      <c r="Y14">
+        <f>W14*100.0869</f>
         <v>225.63411090877582</v>
       </c>
-      <c r="Y14">
+      <c r="Z14">
         <v>230.31890204975423</v>
       </c>
     </row>
-    <row r="18" spans="17:22" x14ac:dyDescent="0.2">
-      <c r="Q18" s="6"/>
+    <row r="18" spans="18:23" x14ac:dyDescent="0.2">
       <c r="R18" s="6"/>
       <c r="S18" s="6"/>
       <c r="T18" s="6"/>
       <c r="U18" s="6"/>
       <c r="V18" s="6"/>
+      <c r="W18" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>